<commit_message>
Publish daily brief and COMEX delivery dashboard with refreshed public data
</commit_message>
<xml_diff>
--- a/全量数据/COMEX金银库存.xlsx
+++ b/全量数据/COMEX金银库存.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMEX金银库存" sheetId="1" r:id="Rbdaf698a563c4510"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人为增添数据" sheetId="2" r:id="R09bb0fe48b6f4eb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMEX金银库存" sheetId="1" r:id="Rdbdd33fcd31b44df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人为增添数据" sheetId="2" r:id="R75fe0a0fdd33473a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -627,6 +627,32 @@
         <x:v>10516.134832069883</x:v>
       </x:c>
     </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="2" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="n">
+        <x:v>460.76121530736117</x:v>
+      </x:c>
+      <x:c r="C9" s="3" t="n">
+        <x:v>54.31510360956826</x:v>
+      </x:c>
+      <x:c r="D9" s="3" t="n">
+        <x:v>261.2251926117063</x:v>
+      </x:c>
+      <x:c r="E9" s="3" t="n">
+        <x:v>721.9864079190676</x:v>
+      </x:c>
+      <x:c r="F9" s="3" t="n">
+        <x:v>3103.910804590023</x:v>
+      </x:c>
+      <x:c r="G9" s="3" t="n">
+        <x:v>7393.460794603999</x:v>
+      </x:c>
+      <x:c r="H9" s="3" t="n">
+        <x:v>10497.37159919402</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -850,6 +876,32 @@
         <x:v>338101585.8674</x:v>
       </x:c>
     </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="2" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="n">
+        <x:v>14813817.062</x:v>
+      </x:c>
+      <x:c r="C9" s="3" t="n">
+        <x:v>1746271.131</x:v>
+      </x:c>
+      <x:c r="D9" s="3" t="n">
+        <x:v>8398584.965</x:v>
+      </x:c>
+      <x:c r="E9" s="3" t="n">
+        <x:v>23212402.027000003</x:v>
+      </x:c>
+      <x:c r="F9" s="3" t="n">
+        <x:v>99793049.64999999</x:v>
+      </x:c>
+      <x:c r="G9" s="3" t="n">
+        <x:v>237705284.27240002</x:v>
+      </x:c>
+      <x:c r="H9" s="3" t="n">
+        <x:v>337498333.9224</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Update dashboard and data
</commit_message>
<xml_diff>
--- a/全量数据/COMEX金银库存.xlsx
+++ b/全量数据/COMEX金银库存.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMEX金银库存" sheetId="1" r:id="Rdbdd33fcd31b44df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人为增添数据" sheetId="2" r:id="R75fe0a0fdd33473a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMEX金银库存" sheetId="1" r:id="R4a44d2ecccef499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人为增添数据" sheetId="2" r:id="Ra3c81dbfc7314018"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -653,6 +653,58 @@
         <x:v>10497.37159919402</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="2" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="n">
+        <x:v>460.76121530736117</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="n">
+        <x:v>54.6268656390628</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="n">
+        <x:v>261.2251926117063</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="n">
+        <x:v>721.9864079190676</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="n">
+        <x:v>3103.910804590023</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="n">
+        <x:v>7393.460794603999</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="n">
+        <x:v>10497.37159919402</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="2" t="d">
+        <x:v>2026-10-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="n">
+        <x:v>461.0729773368558</x:v>
+      </x:c>
+      <x:c r="C11" s="3" t="n">
+        <x:v>54.6268656390628</x:v>
+      </x:c>
+      <x:c r="D11" s="3" t="n">
+        <x:v>260.4230668214093</x:v>
+      </x:c>
+      <x:c r="E11" s="3" t="n">
+        <x:v>721.496044158265</x:v>
+      </x:c>
+      <x:c r="F11" s="3" t="n">
+        <x:v>3104.0681844502137</x:v>
+      </x:c>
+      <x:c r="G11" s="3" t="n">
+        <x:v>7384.181887211812</x:v>
+      </x:c>
+      <x:c r="H11" s="3" t="n">
+        <x:v>10488.250071662025</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -902,6 +954,58 @@
         <x:v>337498333.9224</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="2" t="d">
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="n">
+        <x:v>14813817.062</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="n">
+        <x:v>1756294.513</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="n">
+        <x:v>8398584.965</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="n">
+        <x:v>23212402.027000003</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="n">
+        <x:v>99793049.64999999</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="n">
+        <x:v>237705284.27240002</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="n">
+        <x:v>337498333.9224</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="2" t="d">
+        <x:v>2026-10-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="n">
+        <x:v>14823840.444000002</x:v>
+      </x:c>
+      <x:c r="C11" s="3" t="n">
+        <x:v>1756294.513</x:v>
+      </x:c>
+      <x:c r="D11" s="3" t="n">
+        <x:v>8372796.022000001</x:v>
+      </x:c>
+      <x:c r="E11" s="3" t="n">
+        <x:v>23196636.466000002</x:v>
+      </x:c>
+      <x:c r="F11" s="3" t="n">
+        <x:v>99798109.52999999</x:v>
+      </x:c>
+      <x:c r="G11" s="3" t="n">
+        <x:v>237406960.47240004</x:v>
+      </x:c>
+      <x:c r="H11" s="3" t="n">
+        <x:v>337205070.00240004</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Update dashboard interface and public data for 2026-10-29
</commit_message>
<xml_diff>
--- a/全量数据/COMEX金银库存.xlsx
+++ b/全量数据/COMEX金银库存.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMEX金银库存" sheetId="1" r:id="R4a44d2ecccef499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人为增添数据" sheetId="2" r:id="Ra3c81dbfc7314018"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMEX金银库存" sheetId="1" r:id="Rcb327f94c0a14b88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人为增添数据" sheetId="2" r:id="Rccbc29244f0046f1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -705,6 +705,32 @@
         <x:v>10488.250071662025</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="2" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="n">
+        <x:v>461.23587759762637</x:v>
+      </x:c>
+      <x:c r="C12" s="3" t="n">
+        <x:v>54.6268656390628</x:v>
+      </x:c>
+      <x:c r="D12" s="3" t="n">
+        <x:v>260.5776436051674</x:v>
+      </x:c>
+      <x:c r="E12" s="3" t="n">
+        <x:v>721.8135212027938</x:v>
+      </x:c>
+      <x:c r="F12" s="3" t="n">
+        <x:v>3104.0681844502137</x:v>
+      </x:c>
+      <x:c r="G12" s="3" t="n">
+        <x:v>7363.415850112957</x:v>
+      </x:c>
+      <x:c r="H12" s="3" t="n">
+        <x:v>10467.48403456317</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1006,6 +1032,32 @@
         <x:v>337205070.00240004</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="2" t="d">
+        <x:v>2026-10-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="n">
+        <x:v>14829077.809000002</x:v>
+      </x:c>
+      <x:c r="C12" s="3" t="n">
+        <x:v>1756294.513</x:v>
+      </x:c>
+      <x:c r="D12" s="3" t="n">
+        <x:v>8377765.781000001</x:v>
+      </x:c>
+      <x:c r="E12" s="3" t="n">
+        <x:v>23206843.590000004</x:v>
+      </x:c>
+      <x:c r="F12" s="3" t="n">
+        <x:v>99798109.52999999</x:v>
+      </x:c>
+      <x:c r="G12" s="3" t="n">
+        <x:v>236739316.87640002</x:v>
+      </x:c>
+      <x:c r="H12" s="3" t="n">
+        <x:v>336537426.4064</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Update public dashboard data for 2026-10-30
</commit_message>
<xml_diff>
--- a/全量数据/COMEX金银库存.xlsx
+++ b/全量数据/COMEX金银库存.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMEX金银库存" sheetId="1" r:id="Rcb327f94c0a14b88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人为增添数据" sheetId="2" r:id="Rccbc29244f0046f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMEX金银库存" sheetId="1" r:id="Rf2a2204899fd454f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人为增添数据" sheetId="2" r:id="Rbeb61da6b2714337"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -713,7 +713,7 @@
         <x:v>461.23587759762637</x:v>
       </x:c>
       <x:c r="C12" s="3" t="n">
-        <x:v>54.6268656390628</x:v>
+        <x:v>54.62086559176722</x:v>
       </x:c>
       <x:c r="D12" s="3" t="n">
         <x:v>260.5776436051674</x:v>
@@ -729,6 +729,32 @@
       </x:c>
       <x:c r="H12" s="3" t="n">
         <x:v>10467.48403456317</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2" t="d">
+        <x:v>2026-10-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="n">
+        <x:v>461.23587759762637</x:v>
+      </x:c>
+      <x:c r="C13" s="3" t="n">
+        <x:v>54.62086559176722</x:v>
+      </x:c>
+      <x:c r="D13" s="3" t="n">
+        <x:v>260.56555228407876</x:v>
+      </x:c>
+      <x:c r="E13" s="3" t="n">
+        <x:v>721.8014298817052</x:v>
+      </x:c>
+      <x:c r="F13" s="3" t="n">
+        <x:v>3254.652581508169</x:v>
+      </x:c>
+      <x:c r="G13" s="3" t="n">
+        <x:v>7192.1281216851</x:v>
+      </x:c>
+      <x:c r="H13" s="3" t="n">
+        <x:v>10446.78070319327</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1040,7 +1066,7 @@
         <x:v>14829077.809000002</x:v>
       </x:c>
       <x:c r="C12" s="3" t="n">
-        <x:v>1756294.513</x:v>
+        <x:v>1756101.607</x:v>
       </x:c>
       <x:c r="D12" s="3" t="n">
         <x:v>8377765.781000001</x:v>
@@ -1056,6 +1082,32 @@
       </x:c>
       <x:c r="H12" s="3" t="n">
         <x:v>336537426.4064</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2" t="d">
+        <x:v>2026-10-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="n">
+        <x:v>14829077.809000002</x:v>
+      </x:c>
+      <x:c r="C13" s="3" t="n">
+        <x:v>1756101.607</x:v>
+      </x:c>
+      <x:c r="D13" s="3" t="n">
+        <x:v>8377377.036</x:v>
+      </x:c>
+      <x:c r="E13" s="3" t="n">
+        <x:v>23206454.845000003</x:v>
+      </x:c>
+      <x:c r="F13" s="3" t="n">
+        <x:v>104639510.31699997</x:v>
+      </x:c>
+      <x:c r="G13" s="3" t="n">
+        <x:v>231232288.52940005</x:v>
+      </x:c>
+      <x:c r="H13" s="3" t="n">
+        <x:v>335871798.8464</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Update public dashboard data for 2026-10-31
</commit_message>
<xml_diff>
--- a/全量数据/COMEX金银库存.xlsx
+++ b/全量数据/COMEX金银库存.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMEX金银库存" sheetId="1" r:id="Rf2a2204899fd454f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人为增添数据" sheetId="2" r:id="Rbeb61da6b2714337"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMEX金银库存" sheetId="1" r:id="Rbc910736385f4e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人为增添数据" sheetId="2" r:id="Rc991fb54ed6a42b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -739,7 +739,7 @@
         <x:v>461.23587759762637</x:v>
       </x:c>
       <x:c r="C13" s="3" t="n">
-        <x:v>54.62086559176722</x:v>
+        <x:v>53.439371970183146</x:v>
       </x:c>
       <x:c r="D13" s="3" t="n">
         <x:v>260.56555228407876</x:v>
@@ -755,6 +755,32 @@
       </x:c>
       <x:c r="H13" s="3" t="n">
         <x:v>10446.78070319327</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="n">
+        <x:v>460.6270227469866</x:v>
+      </x:c>
+      <x:c r="C14" s="3" t="n">
+        <x:v>53.439371970183146</x:v>
+      </x:c>
+      <x:c r="D14" s="3" t="n">
+        <x:v>261.09440644190386</x:v>
+      </x:c>
+      <x:c r="E14" s="3" t="n">
+        <x:v>721.7214291888905</x:v>
+      </x:c>
+      <x:c r="F14" s="3" t="n">
+        <x:v>3243.6716662673243</x:v>
+      </x:c>
+      <x:c r="G14" s="3" t="n">
+        <x:v>7199.663504898763</x:v>
+      </x:c>
+      <x:c r="H14" s="3" t="n">
+        <x:v>10443.335171166087</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1092,7 +1118,7 @@
         <x:v>14829077.809000002</x:v>
       </x:c>
       <x:c r="C13" s="3" t="n">
-        <x:v>1756101.607</x:v>
+        <x:v>1718115.705</x:v>
       </x:c>
       <x:c r="D13" s="3" t="n">
         <x:v>8377377.036</x:v>
@@ -1108,6 +1134,32 @@
       </x:c>
       <x:c r="H13" s="3" t="n">
         <x:v>335871798.8464</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="n">
+        <x:v>14809502.671000002</x:v>
+      </x:c>
+      <x:c r="C14" s="3" t="n">
+        <x:v>1718115.705</x:v>
+      </x:c>
+      <x:c r="D14" s="3" t="n">
+        <x:v>8394380.092</x:v>
+      </x:c>
+      <x:c r="E14" s="3" t="n">
+        <x:v>23203882.763000004</x:v>
+      </x:c>
+      <x:c r="F14" s="3" t="n">
+        <x:v>104286465.69399998</x:v>
+      </x:c>
+      <x:c r="G14" s="3" t="n">
+        <x:v>231474556.7254</x:v>
+      </x:c>
+      <x:c r="H14" s="3" t="n">
+        <x:v>335761022.4194</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>